<commit_message>
Firm OS: scale rules-FM to 4 pilot books + iterative water-fill allocation
- make_pilot_books.py: builds the 4 flagship pilot books in one pass (ICICI Pru Large
  Cap, SBI Equity Hybrid, ABSL Flexi Cap, Quant Small Cap) + their daily fact sheets.
- build_rules_v0 upgrades: (1) hybrid/BAF mandates target the middle of their equity
  band (equity_max) so the debt sleeve shows as cash; (2) replace one-shot proportional
  weights with an ITERATIVE WATER-FILL that redistributes leftover from capped names to
  those with headroom under both name + sector caps — fixes large residual cash; (3)
  exempt unknown-sector ("N.A.") names from the sector cap (they aren't one sector).

Result (marked 2026-06-25): ICICI 55 nm/95% eq, SBI 42 nm/72.5% eq, ABSL 70 nm/95%,
Quant 90 nm/95% (was 30% before the fix). Persisted records remain ARM-free.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wkt9GGoBJ36kFJqgCjcrgw
</commit_message>
<xml_diff>
--- a/amc_book/Aditya Birla Sun Life Mutual Fund/Aditya Birla SL Flexi Cap Fund _G_/FACT_SHEET_2026-06-25.xlsx
+++ b/amc_book/Aditya Birla Sun Life Mutual Fund/Aditya Birla SL Flexi Cap Fund _G_/FACT_SHEET_2026-06-25.xlsx
@@ -618,34 +618,34 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3396605</v>
+        <v>3691683</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>1131.3</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>384.2579</v>
+        <v>417.6401</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>1131.3</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>384.2579</v>
+        <v>417.6401</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>1098.1</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>372.9812</v>
+        <v>405.3837</v>
       </c>
       <c r="M6" s="9" t="n">
         <v>3.0234</v>
       </c>
       <c r="N6" s="10" t="n">
-        <v>0.04486</v>
+        <v>0.04875</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>1.4836</v>
+        <v>1.6125</v>
       </c>
     </row>
     <row r="7">
@@ -663,14 +663,14 @@
       <c r="H7" s="11" t="n"/>
       <c r="I7" s="11" t="n"/>
       <c r="J7" s="13" t="n">
-        <v>384.258</v>
+        <v>417.64</v>
       </c>
       <c r="K7" s="11" t="n"/>
       <c r="L7" s="11" t="n"/>
       <c r="M7" s="11" t="n"/>
       <c r="N7" s="11" t="n"/>
       <c r="O7" s="14" t="n">
-        <v>1.48</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="8">
@@ -698,34 +698,34 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2426735</v>
+        <v>2637556</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>2145.3</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>520.6075</v>
+        <v>565.8348999999999</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>2145.3</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>520.6075</v>
+        <v>565.8348999999999</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2122.8</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>515.1473</v>
+        <v>559.9004</v>
       </c>
       <c r="M8" s="9" t="n">
         <v>1.0599</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>0.02131</v>
+        <v>0.02316</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>2.0101</v>
+        <v>2.1847</v>
       </c>
     </row>
     <row r="9">
@@ -753,34 +753,34 @@
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>1113503</v>
+        <v>1210238</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>2616</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>291.2924</v>
+        <v>316.5983</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>2616</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>291.2924</v>
+        <v>316.5983</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>2660</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>296.1918</v>
+        <v>321.9233</v>
       </c>
       <c r="M9" s="9" t="n">
         <v>-1.6541</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>-0.0186</v>
+        <v>-0.02022</v>
       </c>
       <c r="O9" s="9" t="n">
-        <v>1.1247</v>
+        <v>1.2224</v>
       </c>
     </row>
     <row r="10">
@@ -808,34 +808,34 @@
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>892925</v>
+        <v>970497</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>3054</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>272.6993</v>
+        <v>296.3898</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>3054</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>272.6993</v>
+        <v>296.3898</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>3170.5</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>283.1019</v>
+        <v>307.6961</v>
       </c>
       <c r="M10" s="9" t="n">
         <v>-3.6745</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>-0.03869</v>
+        <v>-0.04205</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>1.0529</v>
+        <v>1.1444</v>
       </c>
     </row>
     <row r="11">
@@ -863,25 +863,25 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>3002524</v>
+        <v>3263366</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>619.25</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>185.9313</v>
+        <v>202.0839</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>619.25</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>185.9313</v>
+        <v>202.0839</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>619.2999</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>185.9463</v>
+        <v>202.1002</v>
       </c>
       <c r="M11" s="9" t="n">
         <v>-0.0081</v>
@@ -890,7 +890,7 @@
         <v>-6e-05</v>
       </c>
       <c r="O11" s="9" t="n">
-        <v>0.7179</v>
+        <v>0.7802</v>
       </c>
     </row>
     <row r="12">
@@ -908,14 +908,14 @@
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
       <c r="J12" s="13" t="n">
-        <v>1270.53</v>
+        <v>1380.907</v>
       </c>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="14" t="n">
-        <v>4.91</v>
+        <v>5.33</v>
       </c>
     </row>
     <row r="13">
@@ -943,34 +943,34 @@
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>522615</v>
+        <v>568017</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>9843</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>514.4099</v>
+        <v>559.0991</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>9843</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>514.4099</v>
+        <v>559.0991</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>9750</v>
       </c>
       <c r="L13" s="8" t="n">
-        <v>509.5496</v>
+        <v>553.8166</v>
       </c>
       <c r="M13" s="9" t="n">
         <v>0.9538</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>0.01894</v>
+        <v>0.02059</v>
       </c>
       <c r="O13" s="9" t="n">
-        <v>1.9861</v>
+        <v>2.1587</v>
       </c>
     </row>
     <row r="14">
@@ -998,34 +998,34 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>1090666</v>
+        <v>1185417</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>3182.2</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>347.0717</v>
+        <v>377.2234</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>3182.2</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>347.0717</v>
+        <v>377.2234</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>3064.5</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>334.2346</v>
+        <v>363.271</v>
       </c>
       <c r="M14" s="9" t="n">
         <v>3.8408</v>
       </c>
       <c r="N14" s="10" t="n">
-        <v>0.05147</v>
+        <v>0.05594</v>
       </c>
       <c r="O14" s="9" t="n">
-        <v>1.3401</v>
+        <v>1.4565</v>
       </c>
     </row>
     <row r="15">
@@ -1053,34 +1053,34 @@
         </is>
       </c>
       <c r="F15" s="6" t="n">
-        <v>3413006</v>
+        <v>3709509</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>998.75</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>340.874</v>
+        <v>370.4872</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>998.75</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>340.874</v>
+        <v>370.4872</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>990.1</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>337.9217</v>
+        <v>367.2785</v>
       </c>
       <c r="M15" s="9" t="n">
         <v>0.8736</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>0.0115</v>
+        <v>0.0125</v>
       </c>
       <c r="O15" s="9" t="n">
-        <v>1.3161</v>
+        <v>1.4305</v>
       </c>
     </row>
     <row r="16">
@@ -1108,34 +1108,34 @@
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>180363</v>
+        <v>196031</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>13745</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>247.9089</v>
+        <v>269.4446</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>13745</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>247.9089</v>
+        <v>269.4446</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>13248</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>238.9449</v>
+        <v>259.7019</v>
       </c>
       <c r="M16" s="9" t="n">
         <v>3.7515</v>
       </c>
       <c r="N16" s="10" t="n">
-        <v>0.03591</v>
+        <v>0.03903</v>
       </c>
       <c r="O16" s="9" t="n">
-        <v>0.9572000000000001</v>
+        <v>1.0403</v>
       </c>
     </row>
     <row r="17">
@@ -1153,14 +1153,14 @@
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
       <c r="J17" s="13" t="n">
-        <v>1450.264</v>
+        <v>1576.254</v>
       </c>
       <c r="K17" s="11" t="n"/>
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
       <c r="O17" s="14" t="n">
-        <v>5.6</v>
+        <v>6.09</v>
       </c>
     </row>
     <row r="18">
@@ -1188,34 +1188,34 @@
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>4675933</v>
+        <v>5082151</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>1033.85</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>483.4213</v>
+        <v>525.4182</v>
       </c>
       <c r="I18" s="7" t="n">
         <v>1033.85</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>483.4213</v>
+        <v>525.4182</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>1067.2</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>499.0156</v>
+        <v>542.3672</v>
       </c>
       <c r="M18" s="9" t="n">
         <v>-3.125</v>
       </c>
       <c r="N18" s="10" t="n">
-        <v>-0.05833</v>
+        <v>-0.06339</v>
       </c>
       <c r="O18" s="9" t="n">
-        <v>1.8665</v>
+        <v>2.0286</v>
       </c>
     </row>
     <row r="19">
@@ -1243,34 +1243,34 @@
         </is>
       </c>
       <c r="F19" s="6" t="n">
-        <v>2790139</v>
+        <v>3032531</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>1377.2</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>384.2579</v>
+        <v>417.6402</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>1377.2</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>384.2579</v>
+        <v>417.6402</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>1384.5</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>386.2947</v>
+        <v>419.8539</v>
       </c>
       <c r="M19" s="9" t="n">
         <v>-0.5273</v>
       </c>
       <c r="N19" s="10" t="n">
-        <v>-0.007820000000000001</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="O19" s="9" t="n">
-        <v>1.4836</v>
+        <v>1.6125</v>
       </c>
     </row>
     <row r="20">
@@ -1298,34 +1298,34 @@
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>2724759</v>
+        <v>2961470</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>1387.5</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>378.0603</v>
+        <v>410.904</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>1387.5</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>378.0603</v>
+        <v>410.904</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>1373.6</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>374.2729</v>
+        <v>406.7875</v>
       </c>
       <c r="M20" s="9" t="n">
         <v>1.0119</v>
       </c>
       <c r="N20" s="10" t="n">
-        <v>0.01477</v>
+        <v>0.01605</v>
       </c>
       <c r="O20" s="9" t="n">
-        <v>1.4597</v>
+        <v>1.5865</v>
       </c>
     </row>
     <row r="21">
@@ -1353,34 +1353,34 @@
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>8788927</v>
+        <v>9552459</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>409</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>359.4671</v>
+        <v>390.6956</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>409</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>359.4671</v>
+        <v>390.6956</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>405.95</v>
       </c>
       <c r="L21" s="8" t="n">
-        <v>356.7865</v>
+        <v>387.7821</v>
       </c>
       <c r="M21" s="9" t="n">
         <v>0.7513</v>
       </c>
       <c r="N21" s="10" t="n">
-        <v>0.01043</v>
+        <v>0.01133</v>
       </c>
       <c r="O21" s="9" t="n">
-        <v>1.3879</v>
+        <v>1.5085</v>
       </c>
     </row>
     <row r="22">
@@ -1408,34 +1408,34 @@
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>8989117</v>
+        <v>9770040</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>324.05</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>291.2923</v>
+        <v>316.5981</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>324.05</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>291.2923</v>
+        <v>316.5981</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>325.2</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>292.3261</v>
+        <v>317.7217</v>
       </c>
       <c r="M22" s="9" t="n">
         <v>-0.3536</v>
       </c>
       <c r="N22" s="10" t="n">
-        <v>-0.00398</v>
+        <v>-0.00432</v>
       </c>
       <c r="O22" s="9" t="n">
-        <v>1.1247</v>
+        <v>1.2224</v>
       </c>
     </row>
     <row r="23">
@@ -1463,34 +1463,34 @@
         </is>
       </c>
       <c r="F23" s="6" t="n">
-        <v>3580241</v>
+        <v>3891272</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>796.3</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>285.0946</v>
+        <v>309.862</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>796.3</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>285.0946</v>
+        <v>309.862</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>793.2</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>283.9847</v>
+        <v>308.6557</v>
       </c>
       <c r="M23" s="9" t="n">
         <v>0.3908</v>
       </c>
       <c r="N23" s="10" t="n">
-        <v>0.0043</v>
+        <v>0.00468</v>
       </c>
       <c r="O23" s="9" t="n">
-        <v>1.1008</v>
+        <v>1.1964</v>
       </c>
     </row>
     <row r="24">
@@ -1518,34 +1518,34 @@
         </is>
       </c>
       <c r="F24" s="6" t="n">
-        <v>2549278</v>
+        <v>2770744</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>1045.4</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>266.5015</v>
+        <v>289.6536</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>1045.4</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>266.5015</v>
+        <v>289.6536</v>
       </c>
       <c r="K24" s="7" t="n">
         <v>1034.6</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>263.7483</v>
+        <v>286.6612</v>
       </c>
       <c r="M24" s="9" t="n">
         <v>1.0439</v>
       </c>
       <c r="N24" s="10" t="n">
-        <v>0.01074</v>
+        <v>0.01167</v>
       </c>
       <c r="O24" s="9" t="n">
-        <v>1.029</v>
+        <v>1.1184</v>
       </c>
     </row>
     <row r="25">
@@ -1563,14 +1563,14 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
       <c r="J25" s="13" t="n">
-        <v>2448.095</v>
+        <v>2660.772</v>
       </c>
       <c r="K25" s="11" t="n"/>
       <c r="L25" s="11" t="n"/>
       <c r="M25" s="11" t="n"/>
       <c r="N25" s="11" t="n"/>
       <c r="O25" s="14" t="n">
-        <v>9.449999999999999</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="26">
@@ -1598,34 +1598,34 @@
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>1229897</v>
+        <v>1336743</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3829.8</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>471.026</v>
+        <v>511.9458</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>3829.8</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>471.026</v>
+        <v>511.9458</v>
       </c>
       <c r="K26" s="7" t="n">
         <v>3757.7</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>462.1584</v>
+        <v>502.3079</v>
       </c>
       <c r="M26" s="9" t="n">
         <v>1.9187</v>
       </c>
       <c r="N26" s="10" t="n">
-        <v>0.03489</v>
+        <v>0.03793</v>
       </c>
       <c r="O26" s="9" t="n">
-        <v>1.8186</v>
+        <v>1.9766</v>
       </c>
     </row>
     <row r="27">
@@ -1653,34 +1653,34 @@
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>1163553</v>
+        <v>1264636</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>1384.9</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>161.1405</v>
+        <v>175.1394</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>1384.9</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>161.1405</v>
+        <v>175.1394</v>
       </c>
       <c r="K27" s="7" t="n">
         <v>1359.1</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>158.1385</v>
+        <v>171.8767</v>
       </c>
       <c r="M27" s="9" t="n">
         <v>1.8983</v>
       </c>
       <c r="N27" s="10" t="n">
-        <v>0.01181</v>
+        <v>0.01284</v>
       </c>
       <c r="O27" s="9" t="n">
-        <v>0.6222</v>
+        <v>0.6762</v>
       </c>
     </row>
     <row r="28">
@@ -1698,14 +1698,14 @@
       <c r="H28" s="11" t="n"/>
       <c r="I28" s="11" t="n"/>
       <c r="J28" s="13" t="n">
-        <v>632.167</v>
+        <v>687.085</v>
       </c>
       <c r="K28" s="11" t="n"/>
       <c r="L28" s="11" t="n"/>
       <c r="M28" s="11" t="n"/>
       <c r="N28" s="11" t="n"/>
       <c r="O28" s="14" t="n">
-        <v>2.44</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="29">
@@ -1733,34 +1733,34 @@
         </is>
       </c>
       <c r="F29" s="6" t="n">
-        <v>13495384</v>
+        <v>14667786</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>335.25</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>452.4327</v>
+        <v>491.7375</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>335.25</v>
       </c>
       <c r="J29" s="8" t="n">
-        <v>452.4327</v>
+        <v>491.7375</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>340.65</v>
       </c>
       <c r="L29" s="8" t="n">
-        <v>459.7203</v>
+        <v>499.6581</v>
       </c>
       <c r="M29" s="9" t="n">
         <v>-1.5852</v>
       </c>
       <c r="N29" s="10" t="n">
-        <v>-0.02769</v>
+        <v>-0.0301</v>
       </c>
       <c r="O29" s="9" t="n">
-        <v>1.7469</v>
+        <v>1.8986</v>
       </c>
     </row>
     <row r="30">
@@ -1778,14 +1778,14 @@
       <c r="H30" s="11" t="n"/>
       <c r="I30" s="11" t="n"/>
       <c r="J30" s="13" t="n">
-        <v>452.433</v>
+        <v>491.738</v>
       </c>
       <c r="K30" s="11" t="n"/>
       <c r="L30" s="11" t="n"/>
       <c r="M30" s="11" t="n"/>
       <c r="N30" s="11" t="n"/>
       <c r="O30" s="14" t="n">
-        <v>1.75</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="31">
@@ -1813,34 +1813,34 @@
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>1942607</v>
+        <v>2111370</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3126.6</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>607.3755</v>
+        <v>660.1409</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>3126.6</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>607.3755</v>
+        <v>660.1409</v>
       </c>
       <c r="K31" s="7" t="n">
         <v>3127.9</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>607.628</v>
+        <v>660.4154</v>
       </c>
       <c r="M31" s="9" t="n">
         <v>-0.0416</v>
       </c>
       <c r="N31" s="10" t="n">
-        <v>-0.00098</v>
+        <v>-0.00106</v>
       </c>
       <c r="O31" s="9" t="n">
-        <v>2.3451</v>
+        <v>2.5488</v>
       </c>
     </row>
     <row r="32">
@@ -1858,14 +1858,14 @@
       <c r="H32" s="11" t="n"/>
       <c r="I32" s="11" t="n"/>
       <c r="J32" s="13" t="n">
-        <v>607.375</v>
+        <v>660.141</v>
       </c>
       <c r="K32" s="11" t="n"/>
       <c r="L32" s="11" t="n"/>
       <c r="M32" s="11" t="n"/>
       <c r="N32" s="11" t="n"/>
       <c r="O32" s="14" t="n">
-        <v>2.35</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="33">
@@ -1973,34 +1973,34 @@
         </is>
       </c>
       <c r="F35" s="6" t="n">
-        <v>2296142</v>
+        <v>2495618</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>2645.2</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>607.3755</v>
+        <v>660.1409</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>2645.2</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>607.3755</v>
+        <v>660.1409</v>
       </c>
       <c r="K35" s="7" t="n">
         <v>2667.5</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>612.4959</v>
+        <v>665.7061</v>
       </c>
       <c r="M35" s="9" t="n">
         <v>-0.836</v>
       </c>
       <c r="N35" s="10" t="n">
-        <v>-0.01961</v>
+        <v>-0.02131</v>
       </c>
       <c r="O35" s="9" t="n">
-        <v>2.3451</v>
+        <v>2.5488</v>
       </c>
     </row>
     <row r="36">
@@ -2073,14 +2073,14 @@
       <c r="H37" s="11" t="n"/>
       <c r="I37" s="11" t="n"/>
       <c r="J37" s="13" t="n">
-        <v>686.377</v>
+        <v>739.1420000000001</v>
       </c>
       <c r="K37" s="11" t="n"/>
       <c r="L37" s="11" t="n"/>
       <c r="M37" s="11" t="n"/>
       <c r="N37" s="11" t="n"/>
       <c r="O37" s="14" t="n">
-        <v>2.65</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="38">
@@ -2108,34 +2108,34 @@
         </is>
       </c>
       <c r="F38" s="6" t="n">
-        <v>4802386</v>
+        <v>5219590</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>942.1</v>
       </c>
       <c r="H38" s="8" t="n">
-        <v>452.4328</v>
+        <v>491.7376</v>
       </c>
       <c r="I38" s="7" t="n">
         <v>942.1</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>452.4328</v>
+        <v>491.7376</v>
       </c>
       <c r="K38" s="7" t="n">
         <v>919.45</v>
       </c>
       <c r="L38" s="8" t="n">
-        <v>441.5554</v>
+        <v>479.9152</v>
       </c>
       <c r="M38" s="9" t="n">
         <v>2.4634</v>
       </c>
       <c r="N38" s="10" t="n">
-        <v>0.04303</v>
+        <v>0.04677</v>
       </c>
       <c r="O38" s="9" t="n">
-        <v>1.7469</v>
+        <v>1.8986</v>
       </c>
     </row>
     <row r="39">
@@ -2153,14 +2153,14 @@
       <c r="H39" s="11" t="n"/>
       <c r="I39" s="11" t="n"/>
       <c r="J39" s="13" t="n">
-        <v>452.433</v>
+        <v>491.738</v>
       </c>
       <c r="K39" s="11" t="n"/>
       <c r="L39" s="11" t="n"/>
       <c r="M39" s="11" t="n"/>
       <c r="N39" s="11" t="n"/>
       <c r="O39" s="14" t="n">
-        <v>1.75</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="40">
@@ -2188,34 +2188,34 @@
         </is>
       </c>
       <c r="F40" s="6" t="n">
-        <v>3217310</v>
+        <v>3496812</v>
       </c>
       <c r="G40" s="7" t="n">
         <v>1059.5</v>
       </c>
       <c r="H40" s="8" t="n">
-        <v>340.874</v>
+        <v>370.4872</v>
       </c>
       <c r="I40" s="7" t="n">
         <v>1059.5</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>340.874</v>
+        <v>370.4872</v>
       </c>
       <c r="K40" s="7" t="n">
         <v>1089.7</v>
       </c>
       <c r="L40" s="8" t="n">
-        <v>350.5903</v>
+        <v>381.0476</v>
       </c>
       <c r="M40" s="9" t="n">
         <v>-2.7714</v>
       </c>
       <c r="N40" s="10" t="n">
-        <v>-0.03647</v>
+        <v>-0.03964</v>
       </c>
       <c r="O40" s="9" t="n">
-        <v>1.3161</v>
+        <v>1.4305</v>
       </c>
     </row>
     <row r="41">
@@ -2233,14 +2233,14 @@
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
       <c r="J41" s="13" t="n">
-        <v>340.874</v>
+        <v>370.487</v>
       </c>
       <c r="K41" s="11" t="n"/>
       <c r="L41" s="11" t="n"/>
       <c r="M41" s="11" t="n"/>
       <c r="N41" s="11" t="n"/>
       <c r="O41" s="14" t="n">
-        <v>1.32</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="42">
@@ -2268,34 +2268,34 @@
         </is>
       </c>
       <c r="F42" s="6" t="n">
-        <v>438588</v>
+        <v>476690</v>
       </c>
       <c r="G42" s="7" t="n">
         <v>2684.9</v>
       </c>
       <c r="H42" s="8" t="n">
-        <v>117.7565</v>
+        <v>127.9865</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>2684.9</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>117.7565</v>
+        <v>127.9865</v>
       </c>
       <c r="K42" s="7" t="n">
         <v>2746.8</v>
       </c>
       <c r="L42" s="8" t="n">
-        <v>120.4714</v>
+        <v>130.9372</v>
       </c>
       <c r="M42" s="9" t="n">
         <v>-2.2535</v>
       </c>
       <c r="N42" s="10" t="n">
-        <v>-0.01025</v>
+        <v>-0.01114</v>
       </c>
       <c r="O42" s="9" t="n">
-        <v>0.4547</v>
+        <v>0.4942</v>
       </c>
     </row>
     <row r="43">
@@ -2323,34 +2323,34 @@
         </is>
       </c>
       <c r="F43" s="6" t="n">
-        <v>2135668</v>
+        <v>2321203</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>435.3</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>92.96559999999999</v>
+        <v>101.042</v>
       </c>
       <c r="I43" s="7" t="n">
         <v>435.3</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>92.96559999999999</v>
+        <v>101.042</v>
       </c>
       <c r="K43" s="7" t="n">
         <v>446.05</v>
       </c>
       <c r="L43" s="8" t="n">
-        <v>95.2615</v>
+        <v>103.5373</v>
       </c>
       <c r="M43" s="9" t="n">
         <v>-2.41</v>
       </c>
       <c r="N43" s="10" t="n">
-        <v>-0.00865</v>
+        <v>-0.0094</v>
       </c>
       <c r="O43" s="9" t="n">
-        <v>0.3589</v>
+        <v>0.3901</v>
       </c>
     </row>
     <row r="44">
@@ -2368,14 +2368,14 @@
       <c r="H44" s="11" t="n"/>
       <c r="I44" s="11" t="n"/>
       <c r="J44" s="13" t="n">
-        <v>210.722</v>
+        <v>229.029</v>
       </c>
       <c r="K44" s="11" t="n"/>
       <c r="L44" s="11" t="n"/>
       <c r="M44" s="11" t="n"/>
       <c r="N44" s="11" t="n"/>
       <c r="O44" s="14" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="45">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>INE741K01010</t>
+          <t>INE121A01024</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>CreditAccess Grameen Limited</t>
+          <t>Cholamandalam Investment and Finance Company Limited</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -2403,34 +2403,34 @@
         </is>
       </c>
       <c r="F45" s="6" t="n">
-        <v>3687704</v>
+        <v>3182365</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>1462.3</v>
+        <v>1799.2</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>539.253</v>
+        <v>572.5711</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>1462.3</v>
+        <v>1799.2</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>539.253</v>
+        <v>572.5711</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>1460.3</v>
+        <v>1792.9</v>
       </c>
       <c r="L45" s="8" t="n">
-        <v>538.5154</v>
+        <v>570.5662</v>
       </c>
       <c r="M45" s="9" t="n">
-        <v>0.137</v>
+        <v>0.3514</v>
       </c>
       <c r="N45" s="10" t="n">
-        <v>0.00285</v>
+        <v>0.00777</v>
       </c>
       <c r="O45" s="9" t="n">
-        <v>2.0821</v>
+        <v>2.2107</v>
       </c>
     </row>
     <row r="46">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>INE121A01024</t>
+          <t>INE741K01010</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Cholamandalam Investment and Finance Company Limited</t>
+          <t>CreditAccess Grameen Limited</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -2458,34 +2458,34 @@
         </is>
       </c>
       <c r="F46" s="6" t="n">
-        <v>2927997</v>
+        <v>3687704</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>1799.2</v>
+        <v>1462.3</v>
       </c>
       <c r="H46" s="8" t="n">
-        <v>526.8052</v>
+        <v>539.253</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>1799.2</v>
+        <v>1462.3</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>526.8052</v>
+        <v>539.253</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>1792.9</v>
+        <v>1460.3</v>
       </c>
       <c r="L46" s="8" t="n">
-        <v>524.9606</v>
+        <v>538.5154</v>
       </c>
       <c r="M46" s="9" t="n">
-        <v>0.3514</v>
+        <v>0.137</v>
       </c>
       <c r="N46" s="10" t="n">
-        <v>0.00715</v>
+        <v>0.00285</v>
       </c>
       <c r="O46" s="9" t="n">
-        <v>2.034</v>
+        <v>2.0821</v>
       </c>
     </row>
     <row r="47">
@@ -2513,34 +2513,34 @@
         </is>
       </c>
       <c r="F47" s="6" t="n">
-        <v>8913093</v>
+        <v>9687412</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>299</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>266.5015</v>
+        <v>289.6536</v>
       </c>
       <c r="I47" s="7" t="n">
         <v>299</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>266.5015</v>
+        <v>289.6536</v>
       </c>
       <c r="K47" s="7" t="n">
         <v>296.55</v>
       </c>
       <c r="L47" s="8" t="n">
-        <v>264.3178</v>
+        <v>287.2802</v>
       </c>
       <c r="M47" s="9" t="n">
         <v>0.8262</v>
       </c>
       <c r="N47" s="10" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.00924</v>
       </c>
       <c r="O47" s="9" t="n">
-        <v>1.029</v>
+        <v>1.1184</v>
       </c>
     </row>
     <row r="48">
@@ -2568,34 +2568,34 @@
         </is>
       </c>
       <c r="F48" s="6" t="n">
-        <v>2402678</v>
+        <v>2611409</v>
       </c>
       <c r="G48" s="7" t="n">
         <v>1031.8</v>
       </c>
       <c r="H48" s="8" t="n">
-        <v>247.9083</v>
+        <v>269.4452</v>
       </c>
       <c r="I48" s="7" t="n">
         <v>1031.8</v>
       </c>
       <c r="J48" s="8" t="n">
-        <v>247.9083</v>
+        <v>269.4452</v>
       </c>
       <c r="K48" s="7" t="n">
         <v>1019</v>
       </c>
       <c r="L48" s="8" t="n">
-        <v>244.8329</v>
+        <v>266.1026</v>
       </c>
       <c r="M48" s="9" t="n">
         <v>1.2561</v>
       </c>
       <c r="N48" s="10" t="n">
-        <v>0.01202</v>
+        <v>0.01307</v>
       </c>
       <c r="O48" s="9" t="n">
-        <v>0.9572000000000001</v>
+        <v>1.0403</v>
       </c>
     </row>
     <row r="49">
@@ -2623,34 +2623,34 @@
         </is>
       </c>
       <c r="F49" s="6" t="n">
-        <v>1369776</v>
+        <v>1488774</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>1764.6</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>241.7107</v>
+        <v>262.7091</v>
       </c>
       <c r="I49" s="7" t="n">
         <v>1764.6</v>
       </c>
       <c r="J49" s="8" t="n">
-        <v>241.7107</v>
+        <v>262.7091</v>
       </c>
       <c r="K49" s="7" t="n">
         <v>1780.5</v>
       </c>
       <c r="L49" s="8" t="n">
-        <v>243.8886</v>
+        <v>265.0762</v>
       </c>
       <c r="M49" s="9" t="n">
         <v>-0.893</v>
       </c>
       <c r="N49" s="10" t="n">
-        <v>-0.008330000000000001</v>
+        <v>-0.00906</v>
       </c>
       <c r="O49" s="9" t="n">
-        <v>0.9332</v>
+        <v>1.0143</v>
       </c>
     </row>
     <row r="50">
@@ -2723,14 +2723,14 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="11" t="n"/>
       <c r="J51" s="13" t="n">
-        <v>1986.241</v>
+        <v>2097.694</v>
       </c>
       <c r="K51" s="11" t="n"/>
       <c r="L51" s="11" t="n"/>
       <c r="M51" s="11" t="n"/>
       <c r="N51" s="11" t="n"/>
       <c r="O51" s="14" t="n">
-        <v>7.67</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="52">
@@ -2758,34 +2758,34 @@
         </is>
       </c>
       <c r="F52" s="6" t="n">
-        <v>2715075</v>
+        <v>2950945</v>
       </c>
       <c r="G52" s="7" t="n">
         <v>1689.2</v>
       </c>
       <c r="H52" s="8" t="n">
-        <v>458.6305</v>
+        <v>498.4736</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>1689.2</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>458.6305</v>
+        <v>498.4736</v>
       </c>
       <c r="K52" s="7" t="n">
         <v>1656.0784</v>
       </c>
       <c r="L52" s="8" t="n">
-        <v>449.6377</v>
+        <v>488.6996</v>
       </c>
       <c r="M52" s="9" t="n">
         <v>2</v>
       </c>
       <c r="N52" s="10" t="n">
-        <v>0.03542</v>
+        <v>0.03849</v>
       </c>
       <c r="O52" s="9" t="n">
-        <v>1.7708</v>
+        <v>1.9246</v>
       </c>
     </row>
     <row r="53">
@@ -2813,34 +2813,34 @@
         </is>
       </c>
       <c r="F53" s="6" t="n">
-        <v>411161</v>
+        <v>446880</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>8592</v>
       </c>
       <c r="H53" s="8" t="n">
-        <v>353.2695</v>
+        <v>383.9593</v>
       </c>
       <c r="I53" s="7" t="n">
         <v>8592</v>
       </c>
       <c r="J53" s="8" t="n">
-        <v>353.2695</v>
+        <v>383.9593</v>
       </c>
       <c r="K53" s="7" t="n">
         <v>8573.5</v>
       </c>
       <c r="L53" s="8" t="n">
-        <v>352.5089</v>
+        <v>383.1326</v>
       </c>
       <c r="M53" s="9" t="n">
         <v>0.2158</v>
       </c>
       <c r="N53" s="10" t="n">
-        <v>0.00294</v>
+        <v>0.0032</v>
       </c>
       <c r="O53" s="9" t="n">
-        <v>1.364</v>
+        <v>1.4825</v>
       </c>
     </row>
     <row r="54">
@@ -2913,14 +2913,14 @@
       <c r="H55" s="11" t="n"/>
       <c r="I55" s="11" t="n"/>
       <c r="J55" s="13" t="n">
-        <v>989.5549999999999</v>
+        <v>1060.088</v>
       </c>
       <c r="K55" s="11" t="n"/>
       <c r="L55" s="11" t="n"/>
       <c r="M55" s="11" t="n"/>
       <c r="N55" s="11" t="n"/>
       <c r="O55" s="14" t="n">
-        <v>3.82</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="56">
@@ -3028,34 +3028,34 @@
         </is>
       </c>
       <c r="F58" s="6" t="n">
-        <v>3320740</v>
+        <v>3609227</v>
       </c>
       <c r="G58" s="7" t="n">
         <v>1437.1</v>
       </c>
       <c r="H58" s="8" t="n">
-        <v>477.2235</v>
+        <v>518.682</v>
       </c>
       <c r="I58" s="7" t="n">
         <v>1437.1</v>
       </c>
       <c r="J58" s="8" t="n">
-        <v>477.2235</v>
+        <v>518.682</v>
       </c>
       <c r="K58" s="7" t="n">
         <v>1461.6</v>
       </c>
       <c r="L58" s="8" t="n">
-        <v>485.3594</v>
+        <v>527.5246</v>
       </c>
       <c r="M58" s="9" t="n">
         <v>-1.6762</v>
       </c>
       <c r="N58" s="10" t="n">
-        <v>-0.03089</v>
+        <v>-0.03357</v>
       </c>
       <c r="O58" s="9" t="n">
-        <v>1.8426</v>
+        <v>2.0026</v>
       </c>
     </row>
     <row r="59">
@@ -3083,34 +3083,34 @@
         </is>
       </c>
       <c r="F59" s="6" t="n">
-        <v>3452431</v>
+        <v>3752359</v>
       </c>
       <c r="G59" s="7" t="n">
         <v>1041.2</v>
       </c>
       <c r="H59" s="8" t="n">
-        <v>359.4671</v>
+        <v>390.6956</v>
       </c>
       <c r="I59" s="7" t="n">
         <v>1041.2</v>
       </c>
       <c r="J59" s="8" t="n">
-        <v>359.4671</v>
+        <v>390.6956</v>
       </c>
       <c r="K59" s="7" t="n">
         <v>1056.6</v>
       </c>
       <c r="L59" s="8" t="n">
-        <v>364.7839</v>
+        <v>396.4743</v>
       </c>
       <c r="M59" s="9" t="n">
         <v>-1.4575</v>
       </c>
       <c r="N59" s="10" t="n">
-        <v>-0.02023</v>
+        <v>-0.02199</v>
       </c>
       <c r="O59" s="9" t="n">
-        <v>1.3879</v>
+        <v>1.5085</v>
       </c>
     </row>
     <row r="60">
@@ -3138,34 +3138,34 @@
         </is>
       </c>
       <c r="F60" s="6" t="n">
-        <v>588856</v>
+        <v>640012</v>
       </c>
       <c r="G60" s="7" t="n">
         <v>4841.5</v>
       </c>
       <c r="H60" s="8" t="n">
-        <v>285.0946</v>
+        <v>309.8618</v>
       </c>
       <c r="I60" s="7" t="n">
         <v>4841.5</v>
       </c>
       <c r="J60" s="8" t="n">
-        <v>285.0946</v>
+        <v>309.8618</v>
       </c>
       <c r="K60" s="7" t="n">
         <v>4928.5</v>
       </c>
       <c r="L60" s="8" t="n">
-        <v>290.2177</v>
+        <v>315.4299</v>
       </c>
       <c r="M60" s="9" t="n">
         <v>-1.7652</v>
       </c>
       <c r="N60" s="10" t="n">
-        <v>-0.01943</v>
+        <v>-0.02112</v>
       </c>
       <c r="O60" s="9" t="n">
-        <v>1.1008</v>
+        <v>1.1964</v>
       </c>
     </row>
     <row r="61">
@@ -3193,34 +3193,34 @@
         </is>
       </c>
       <c r="F61" s="6" t="n">
-        <v>1463981</v>
+        <v>1591164</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>1100.7</v>
       </c>
       <c r="H61" s="8" t="n">
-        <v>161.1404</v>
+        <v>175.1394</v>
       </c>
       <c r="I61" s="7" t="n">
         <v>1100.7</v>
       </c>
       <c r="J61" s="8" t="n">
-        <v>161.1404</v>
+        <v>175.1394</v>
       </c>
       <c r="K61" s="7" t="n">
         <v>1113.9</v>
       </c>
       <c r="L61" s="8" t="n">
-        <v>163.0728</v>
+        <v>177.2398</v>
       </c>
       <c r="M61" s="9" t="n">
         <v>-1.185</v>
       </c>
       <c r="N61" s="10" t="n">
-        <v>-0.00737</v>
+        <v>-0.00801</v>
       </c>
       <c r="O61" s="9" t="n">
-        <v>0.6222</v>
+        <v>0.6762</v>
       </c>
     </row>
     <row r="62">
@@ -3238,14 +3238,14 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="11" t="n"/>
       <c r="J62" s="13" t="n">
-        <v>1282.926</v>
+        <v>1394.379</v>
       </c>
       <c r="K62" s="11" t="n"/>
       <c r="L62" s="11" t="n"/>
       <c r="M62" s="11" t="n"/>
       <c r="N62" s="11" t="n"/>
       <c r="O62" s="14" t="n">
-        <v>4.95</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="63">
@@ -3273,34 +3273,34 @@
         </is>
       </c>
       <c r="F63" s="6" t="n">
-        <v>78641</v>
+        <v>85473</v>
       </c>
       <c r="G63" s="7" t="n">
         <v>39405</v>
       </c>
       <c r="H63" s="8" t="n">
-        <v>309.8849</v>
+        <v>336.8064</v>
       </c>
       <c r="I63" s="7" t="n">
         <v>39405</v>
       </c>
       <c r="J63" s="8" t="n">
-        <v>309.8849</v>
+        <v>336.8064</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>39015</v>
       </c>
       <c r="L63" s="8" t="n">
-        <v>306.8179</v>
+        <v>333.4729</v>
       </c>
       <c r="M63" s="9" t="n">
         <v>0.9996</v>
       </c>
       <c r="N63" s="10" t="n">
-        <v>0.01196</v>
+        <v>0.013</v>
       </c>
       <c r="O63" s="9" t="n">
-        <v>1.1965</v>
+        <v>1.3004</v>
       </c>
     </row>
     <row r="64">
@@ -3318,14 +3318,14 @@
       <c r="H64" s="11" t="n"/>
       <c r="I64" s="11" t="n"/>
       <c r="J64" s="13" t="n">
-        <v>309.885</v>
+        <v>336.806</v>
       </c>
       <c r="K64" s="11" t="n"/>
       <c r="L64" s="11" t="n"/>
       <c r="M64" s="11" t="n"/>
       <c r="N64" s="11" t="n"/>
       <c r="O64" s="14" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="65">
@@ -3353,34 +3353,34 @@
         </is>
       </c>
       <c r="F65" s="6" t="n">
-        <v>3705592</v>
+        <v>4027513</v>
       </c>
       <c r="G65" s="7" t="n">
         <v>1455.1</v>
       </c>
       <c r="H65" s="8" t="n">
-        <v>539.2007</v>
+        <v>586.0434</v>
       </c>
       <c r="I65" s="7" t="n">
         <v>1455.1</v>
       </c>
       <c r="J65" s="8" t="n">
-        <v>539.2007</v>
+        <v>586.0434</v>
       </c>
       <c r="K65" s="7" t="n">
         <v>1406</v>
       </c>
       <c r="L65" s="8" t="n">
-        <v>521.0062</v>
+        <v>566.2683</v>
       </c>
       <c r="M65" s="9" t="n">
         <v>3.4922</v>
       </c>
       <c r="N65" s="10" t="n">
-        <v>0.0727</v>
+        <v>0.07902000000000001</v>
       </c>
       <c r="O65" s="9" t="n">
-        <v>2.0819</v>
+        <v>2.2627</v>
       </c>
     </row>
     <row r="66">
@@ -3408,34 +3408,34 @@
         </is>
       </c>
       <c r="F66" s="6" t="n">
-        <v>2117129</v>
+        <v>2301053</v>
       </c>
       <c r="G66" s="7" t="n">
         <v>2488.3</v>
       </c>
       <c r="H66" s="8" t="n">
-        <v>526.8052</v>
+        <v>572.571</v>
       </c>
       <c r="I66" s="7" t="n">
         <v>2488.3</v>
       </c>
       <c r="J66" s="8" t="n">
-        <v>526.8052</v>
+        <v>572.571</v>
       </c>
       <c r="K66" s="7" t="n">
         <v>2438</v>
       </c>
       <c r="L66" s="8" t="n">
-        <v>516.1561</v>
+        <v>560.9967</v>
       </c>
       <c r="M66" s="9" t="n">
         <v>2.0632</v>
       </c>
       <c r="N66" s="10" t="n">
-        <v>0.04197</v>
+        <v>0.04561</v>
       </c>
       <c r="O66" s="9" t="n">
-        <v>2.034</v>
+        <v>2.2107</v>
       </c>
     </row>
     <row r="67">
@@ -3463,34 +3463,34 @@
         </is>
       </c>
       <c r="F67" s="6" t="n">
-        <v>3251203</v>
+        <v>3533648</v>
       </c>
       <c r="G67" s="7" t="n">
         <v>1486.9</v>
       </c>
       <c r="H67" s="8" t="n">
-        <v>483.4214</v>
+        <v>525.4181</v>
       </c>
       <c r="I67" s="7" t="n">
         <v>1486.9</v>
       </c>
       <c r="J67" s="8" t="n">
-        <v>483.4214</v>
+        <v>525.4181</v>
       </c>
       <c r="K67" s="7" t="n">
         <v>1536.7</v>
       </c>
       <c r="L67" s="8" t="n">
-        <v>499.6124</v>
+        <v>543.0157</v>
       </c>
       <c r="M67" s="9" t="n">
         <v>-3.2407</v>
       </c>
       <c r="N67" s="10" t="n">
-        <v>-0.06049</v>
+        <v>-0.06574000000000001</v>
       </c>
       <c r="O67" s="9" t="n">
-        <v>1.8665</v>
+        <v>2.0286</v>
       </c>
     </row>
     <row r="68">
@@ -3518,34 +3518,34 @@
         </is>
       </c>
       <c r="F68" s="6" t="n">
-        <v>626142</v>
+        <v>680538</v>
       </c>
       <c r="G68" s="7" t="n">
         <v>5642</v>
       </c>
       <c r="H68" s="8" t="n">
-        <v>353.2693</v>
+        <v>383.9595</v>
       </c>
       <c r="I68" s="7" t="n">
         <v>5642</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>353.2693</v>
+        <v>383.9595</v>
       </c>
       <c r="K68" s="7" t="n">
         <v>5555.5</v>
       </c>
       <c r="L68" s="8" t="n">
-        <v>347.8532</v>
+        <v>378.0729</v>
       </c>
       <c r="M68" s="9" t="n">
         <v>1.557</v>
       </c>
       <c r="N68" s="10" t="n">
-        <v>0.02124</v>
+        <v>0.02308</v>
       </c>
       <c r="O68" s="9" t="n">
-        <v>1.364</v>
+        <v>1.4825</v>
       </c>
     </row>
     <row r="69">
@@ -3628,34 +3628,34 @@
         </is>
       </c>
       <c r="F70" s="6" t="n">
-        <v>1174921</v>
+        <v>1276992</v>
       </c>
       <c r="G70" s="7" t="n">
         <v>1793.5</v>
       </c>
       <c r="H70" s="8" t="n">
-        <v>210.7221</v>
+        <v>229.0285</v>
       </c>
       <c r="I70" s="7" t="n">
         <v>1793.5</v>
       </c>
       <c r="J70" s="8" t="n">
-        <v>210.7221</v>
+        <v>229.0285</v>
       </c>
       <c r="K70" s="7" t="n">
         <v>1826.2</v>
       </c>
       <c r="L70" s="8" t="n">
-        <v>214.5641</v>
+        <v>233.2043</v>
       </c>
       <c r="M70" s="9" t="n">
         <v>-1.7906</v>
       </c>
       <c r="N70" s="10" t="n">
-        <v>-0.01457</v>
+        <v>-0.01583</v>
       </c>
       <c r="O70" s="9" t="n">
-        <v>0.8136</v>
+        <v>0.8843</v>
       </c>
     </row>
     <row r="71">
@@ -3673,14 +3673,14 @@
       <c r="H71" s="11" t="n"/>
       <c r="I71" s="11" t="n"/>
       <c r="J71" s="13" t="n">
-        <v>2358.563</v>
+        <v>2542.164</v>
       </c>
       <c r="K71" s="11" t="n"/>
       <c r="L71" s="11" t="n"/>
       <c r="M71" s="11" t="n"/>
       <c r="N71" s="11" t="n"/>
       <c r="O71" s="14" t="n">
-        <v>9.109999999999999</v>
+        <v>9.81</v>
       </c>
     </row>
     <row r="72">
@@ -3708,34 +3708,34 @@
         </is>
       </c>
       <c r="F72" s="6" t="n">
-        <v>1674502</v>
+        <v>1819974</v>
       </c>
       <c r="G72" s="7" t="n">
         <v>1813.6</v>
       </c>
       <c r="H72" s="8" t="n">
-        <v>303.6877</v>
+        <v>330.0705</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>1813.6</v>
       </c>
       <c r="J72" s="8" t="n">
-        <v>303.6877</v>
+        <v>330.0705</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>1821.1</v>
       </c>
       <c r="L72" s="8" t="n">
-        <v>304.9436</v>
+        <v>331.4355</v>
       </c>
       <c r="M72" s="9" t="n">
         <v>-0.4118</v>
       </c>
       <c r="N72" s="10" t="n">
-        <v>-0.00483</v>
+        <v>-0.00525</v>
       </c>
       <c r="O72" s="9" t="n">
-        <v>1.1725</v>
+        <v>1.2744</v>
       </c>
     </row>
     <row r="73">
@@ -3763,34 +3763,34 @@
         </is>
       </c>
       <c r="F73" s="6" t="n">
-        <v>1669393</v>
+        <v>1814420</v>
       </c>
       <c r="G73" s="7" t="n">
         <v>1744.9</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>291.2924</v>
+        <v>316.5981</v>
       </c>
       <c r="I73" s="7" t="n">
         <v>1744.9</v>
       </c>
       <c r="J73" s="8" t="n">
-        <v>291.2924</v>
+        <v>316.5981</v>
       </c>
       <c r="K73" s="7" t="n">
         <v>1767.7</v>
       </c>
       <c r="L73" s="8" t="n">
-        <v>295.0986</v>
+        <v>320.735</v>
       </c>
       <c r="M73" s="9" t="n">
         <v>-1.2898</v>
       </c>
       <c r="N73" s="10" t="n">
-        <v>-0.01451</v>
+        <v>-0.01577</v>
       </c>
       <c r="O73" s="9" t="n">
-        <v>1.1247</v>
+        <v>1.2224</v>
       </c>
     </row>
     <row r="74">
@@ -3818,34 +3818,34 @@
         </is>
       </c>
       <c r="F74" s="6" t="n">
-        <v>615386</v>
+        <v>668848</v>
       </c>
       <c r="G74" s="7" t="n">
         <v>1611.4</v>
       </c>
       <c r="H74" s="8" t="n">
-        <v>99.16330000000001</v>
+        <v>107.7782</v>
       </c>
       <c r="I74" s="7" t="n">
         <v>1611.4</v>
       </c>
       <c r="J74" s="8" t="n">
-        <v>99.16330000000001</v>
+        <v>107.7782</v>
       </c>
       <c r="K74" s="7" t="n">
         <v>1662.3</v>
       </c>
       <c r="L74" s="8" t="n">
-        <v>102.2956</v>
+        <v>111.1826</v>
       </c>
       <c r="M74" s="9" t="n">
         <v>-3.062</v>
       </c>
       <c r="N74" s="10" t="n">
-        <v>-0.01172</v>
+        <v>-0.01274</v>
       </c>
       <c r="O74" s="9" t="n">
-        <v>0.3829</v>
+        <v>0.4161</v>
       </c>
     </row>
     <row r="75">
@@ -3863,14 +3863,14 @@
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="11" t="n"/>
       <c r="J75" s="13" t="n">
-        <v>694.143</v>
+        <v>754.447</v>
       </c>
       <c r="K75" s="11" t="n"/>
       <c r="L75" s="11" t="n"/>
       <c r="M75" s="11" t="n"/>
       <c r="N75" s="11" t="n"/>
       <c r="O75" s="14" t="n">
-        <v>2.68</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="76">
@@ -3898,34 +3898,34 @@
         </is>
       </c>
       <c r="F76" s="6" t="n">
-        <v>4876502</v>
+        <v>5300145</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>953.2</v>
       </c>
       <c r="H76" s="8" t="n">
-        <v>464.8282</v>
+        <v>505.2098</v>
       </c>
       <c r="I76" s="7" t="n">
         <v>953.2</v>
       </c>
       <c r="J76" s="8" t="n">
-        <v>464.8282</v>
+        <v>505.2098</v>
       </c>
       <c r="K76" s="7" t="n">
         <v>976.6</v>
       </c>
       <c r="L76" s="8" t="n">
-        <v>476.2392</v>
+        <v>517.6122</v>
       </c>
       <c r="M76" s="9" t="n">
         <v>-2.3961</v>
       </c>
       <c r="N76" s="10" t="n">
-        <v>-0.043</v>
+        <v>-0.04674</v>
       </c>
       <c r="O76" s="9" t="n">
-        <v>1.7947</v>
+        <v>1.9506</v>
       </c>
     </row>
     <row r="77">
@@ -3943,14 +3943,14 @@
       <c r="H77" s="11" t="n"/>
       <c r="I77" s="11" t="n"/>
       <c r="J77" s="13" t="n">
-        <v>464.828</v>
+        <v>505.21</v>
       </c>
       <c r="K77" s="11" t="n"/>
       <c r="L77" s="11" t="n"/>
       <c r="M77" s="11" t="n"/>
       <c r="N77" s="11" t="n"/>
       <c r="O77" s="14" t="n">
-        <v>1.79</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="78">
@@ -3978,34 +3978,34 @@
         </is>
       </c>
       <c r="F78" s="6" t="n">
-        <v>1976845</v>
+        <v>2148582</v>
       </c>
       <c r="G78" s="7" t="n">
         <v>1034.6</v>
       </c>
       <c r="H78" s="8" t="n">
-        <v>204.5244</v>
+        <v>222.2923</v>
       </c>
       <c r="I78" s="7" t="n">
         <v>1034.6</v>
       </c>
       <c r="J78" s="8" t="n">
-        <v>204.5244</v>
+        <v>222.2923</v>
       </c>
       <c r="K78" s="7" t="n">
         <v>1020.5</v>
       </c>
       <c r="L78" s="8" t="n">
-        <v>201.737</v>
+        <v>219.2628</v>
       </c>
       <c r="M78" s="9" t="n">
         <v>1.3817</v>
       </c>
       <c r="N78" s="10" t="n">
-        <v>0.01091</v>
+        <v>0.01186</v>
       </c>
       <c r="O78" s="9" t="n">
-        <v>0.7897</v>
+        <v>0.8583</v>
       </c>
     </row>
     <row r="79">
@@ -4023,14 +4023,14 @@
       <c r="H79" s="11" t="n"/>
       <c r="I79" s="11" t="n"/>
       <c r="J79" s="13" t="n">
-        <v>204.524</v>
+        <v>222.292</v>
       </c>
       <c r="K79" s="11" t="n"/>
       <c r="L79" s="11" t="n"/>
       <c r="M79" s="11" t="n"/>
       <c r="N79" s="11" t="n"/>
       <c r="O79" s="14" t="n">
-        <v>0.79</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="80">
@@ -4058,34 +4058,34 @@
         </is>
       </c>
       <c r="F80" s="6" t="n">
-        <v>2303981</v>
+        <v>2504138</v>
       </c>
       <c r="G80" s="7" t="n">
         <v>1318.1</v>
       </c>
       <c r="H80" s="8" t="n">
-        <v>303.6877</v>
+        <v>330.0704</v>
       </c>
       <c r="I80" s="7" t="n">
         <v>1318.1</v>
       </c>
       <c r="J80" s="8" t="n">
-        <v>303.6877</v>
+        <v>330.0704</v>
       </c>
       <c r="K80" s="7" t="n">
         <v>1313.6</v>
       </c>
       <c r="L80" s="8" t="n">
-        <v>302.6509</v>
+        <v>328.9436</v>
       </c>
       <c r="M80" s="9" t="n">
         <v>0.3426</v>
       </c>
       <c r="N80" s="10" t="n">
-        <v>0.00402</v>
+        <v>0.00437</v>
       </c>
       <c r="O80" s="9" t="n">
-        <v>1.1725</v>
+        <v>1.2744</v>
       </c>
     </row>
     <row r="81">
@@ -4103,14 +4103,14 @@
       <c r="H81" s="11" t="n"/>
       <c r="I81" s="11" t="n"/>
       <c r="J81" s="13" t="n">
-        <v>303.688</v>
+        <v>330.07</v>
       </c>
       <c r="K81" s="11" t="n"/>
       <c r="L81" s="11" t="n"/>
       <c r="M81" s="11" t="n"/>
       <c r="N81" s="11" t="n"/>
       <c r="O81" s="14" t="n">
-        <v>1.17</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="82">
@@ -4138,34 +4138,34 @@
         </is>
       </c>
       <c r="F82" s="6" t="n">
-        <v>6427977</v>
+        <v>6796196</v>
       </c>
       <c r="G82" s="7" t="n">
         <v>761.7</v>
       </c>
       <c r="H82" s="8" t="n">
-        <v>489.619</v>
+        <v>517.6662</v>
       </c>
       <c r="I82" s="7" t="n">
         <v>761.7</v>
       </c>
       <c r="J82" s="8" t="n">
-        <v>489.619</v>
+        <v>517.6662</v>
       </c>
       <c r="K82" s="7" t="n">
         <v>767.0859</v>
       </c>
       <c r="L82" s="8" t="n">
-        <v>493.081</v>
+        <v>521.3266</v>
       </c>
       <c r="M82" s="9" t="n">
         <v>-0.7020999999999999</v>
       </c>
       <c r="N82" s="10" t="n">
-        <v>-0.01327</v>
+        <v>-0.01403</v>
       </c>
       <c r="O82" s="9" t="n">
-        <v>1.8904</v>
+        <v>1.9987</v>
       </c>
     </row>
     <row r="83">
@@ -4174,12 +4174,12 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>INE044A01036</t>
+          <t>INE570L01029</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>SAI Life Sciences Ltd</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
@@ -4193,34 +4193,34 @@
         </is>
       </c>
       <c r="F83" s="6" t="n">
-        <v>1663547</v>
+        <v>2757771</v>
       </c>
       <c r="G83" s="7" t="n">
-        <v>1862.8</v>
+        <v>1221.3</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>309.8855</v>
+        <v>336.8066</v>
       </c>
       <c r="I83" s="7" t="n">
-        <v>1862.8</v>
+        <v>1221.3</v>
       </c>
       <c r="J83" s="8" t="n">
-        <v>309.8855</v>
+        <v>336.8066</v>
       </c>
       <c r="K83" s="7" t="n">
-        <v>1874.4</v>
+        <v>1205</v>
       </c>
       <c r="L83" s="8" t="n">
-        <v>311.8152</v>
+        <v>332.3114</v>
       </c>
       <c r="M83" s="9" t="n">
-        <v>-0.6189</v>
+        <v>1.3527</v>
       </c>
       <c r="N83" s="10" t="n">
-        <v>-0.00741</v>
+        <v>0.01759</v>
       </c>
       <c r="O83" s="9" t="n">
-        <v>1.1965</v>
+        <v>1.3004</v>
       </c>
     </row>
     <row r="84">
@@ -4229,12 +4229,12 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>INE570L01029</t>
+          <t>INE044A01036</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>SAI Life Sciences Ltd</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
@@ -4248,34 +4248,34 @@
         </is>
       </c>
       <c r="F84" s="6" t="n">
-        <v>2537341</v>
+        <v>1808066</v>
       </c>
       <c r="G84" s="7" t="n">
-        <v>1221.3</v>
+        <v>1862.8</v>
       </c>
       <c r="H84" s="8" t="n">
-        <v>309.8855</v>
+        <v>336.8065</v>
       </c>
       <c r="I84" s="7" t="n">
-        <v>1221.3</v>
+        <v>1862.8</v>
       </c>
       <c r="J84" s="8" t="n">
-        <v>309.8855</v>
+        <v>336.8065</v>
       </c>
       <c r="K84" s="7" t="n">
-        <v>1205</v>
+        <v>1874.4</v>
       </c>
       <c r="L84" s="8" t="n">
-        <v>305.7496</v>
+        <v>338.9039</v>
       </c>
       <c r="M84" s="9" t="n">
-        <v>1.3527</v>
+        <v>-0.6189</v>
       </c>
       <c r="N84" s="10" t="n">
-        <v>0.01619</v>
+        <v>-0.00805</v>
       </c>
       <c r="O84" s="9" t="n">
-        <v>1.1965</v>
+        <v>1.3004</v>
       </c>
     </row>
     <row r="85">
@@ -4303,34 +4303,34 @@
         </is>
       </c>
       <c r="F85" s="6" t="n">
-        <v>981646</v>
+        <v>1066926</v>
       </c>
       <c r="G85" s="7" t="n">
         <v>2462.3</v>
       </c>
       <c r="H85" s="8" t="n">
-        <v>241.7107</v>
+        <v>262.7092</v>
       </c>
       <c r="I85" s="7" t="n">
         <v>2462.3</v>
       </c>
       <c r="J85" s="8" t="n">
-        <v>241.7107</v>
+        <v>262.7092</v>
       </c>
       <c r="K85" s="7" t="n">
         <v>2483</v>
       </c>
       <c r="L85" s="8" t="n">
-        <v>243.7427</v>
+        <v>264.9177</v>
       </c>
       <c r="M85" s="9" t="n">
         <v>-0.8337</v>
       </c>
       <c r="N85" s="10" t="n">
-        <v>-0.00778</v>
+        <v>-0.008460000000000001</v>
       </c>
       <c r="O85" s="9" t="n">
-        <v>0.9332</v>
+        <v>1.0143</v>
       </c>
     </row>
     <row r="86">
@@ -4413,34 +4413,34 @@
         </is>
       </c>
       <c r="F87" s="6" t="n">
-        <v>1234762</v>
+        <v>1342031</v>
       </c>
       <c r="G87" s="7" t="n">
         <v>1556</v>
       </c>
       <c r="H87" s="8" t="n">
-        <v>192.129</v>
+        <v>208.82</v>
       </c>
       <c r="I87" s="7" t="n">
         <v>1556</v>
       </c>
       <c r="J87" s="8" t="n">
-        <v>192.129</v>
+        <v>208.82</v>
       </c>
       <c r="K87" s="7" t="n">
         <v>1564</v>
       </c>
       <c r="L87" s="8" t="n">
-        <v>193.1168</v>
+        <v>209.8936</v>
       </c>
       <c r="M87" s="9" t="n">
         <v>-0.5115</v>
       </c>
       <c r="N87" s="10" t="n">
-        <v>-0.00379</v>
+        <v>-0.00412</v>
       </c>
       <c r="O87" s="9" t="n">
-        <v>0.7418</v>
+        <v>0.8063</v>
       </c>
     </row>
     <row r="88">
@@ -4458,14 +4458,14 @@
       <c r="H88" s="11" t="n"/>
       <c r="I88" s="11" t="n"/>
       <c r="J88" s="13" t="n">
-        <v>1771.552</v>
+        <v>1891.131</v>
       </c>
       <c r="K88" s="11" t="n"/>
       <c r="L88" s="11" t="n"/>
       <c r="M88" s="11" t="n"/>
       <c r="N88" s="11" t="n"/>
       <c r="O88" s="14" t="n">
-        <v>6.84</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="89">
@@ -4573,34 +4573,34 @@
         </is>
       </c>
       <c r="F91" s="6" t="n">
-        <v>11935066</v>
+        <v>12971916</v>
       </c>
       <c r="G91" s="7" t="n">
         <v>508.9</v>
       </c>
       <c r="H91" s="8" t="n">
-        <v>607.3755</v>
+        <v>660.1408</v>
       </c>
       <c r="I91" s="7" t="n">
         <v>508.9</v>
       </c>
       <c r="J91" s="8" t="n">
-        <v>607.3755</v>
+        <v>660.1408</v>
       </c>
       <c r="K91" s="7" t="n">
         <v>516.35</v>
       </c>
       <c r="L91" s="8" t="n">
-        <v>616.2671</v>
+        <v>669.8049</v>
       </c>
       <c r="M91" s="9" t="n">
         <v>-1.4428</v>
       </c>
       <c r="N91" s="10" t="n">
-        <v>-0.03384</v>
+        <v>-0.03677</v>
       </c>
       <c r="O91" s="9" t="n">
-        <v>2.3451</v>
+        <v>2.5488</v>
       </c>
     </row>
     <row r="92">
@@ -4628,34 +4628,34 @@
         </is>
       </c>
       <c r="F92" s="6" t="n">
-        <v>938041</v>
+        <v>1019533</v>
       </c>
       <c r="G92" s="7" t="n">
         <v>4294.6</v>
       </c>
       <c r="H92" s="8" t="n">
-        <v>402.8511</v>
+        <v>437.8486</v>
       </c>
       <c r="I92" s="7" t="n">
         <v>4294.6</v>
       </c>
       <c r="J92" s="8" t="n">
-        <v>402.8511</v>
+        <v>437.8486</v>
       </c>
       <c r="K92" s="7" t="n">
         <v>4336</v>
       </c>
       <c r="L92" s="8" t="n">
-        <v>406.7346</v>
+        <v>442.0695</v>
       </c>
       <c r="M92" s="9" t="n">
         <v>-0.9548</v>
       </c>
       <c r="N92" s="10" t="n">
-        <v>-0.01485</v>
+        <v>-0.01614</v>
       </c>
       <c r="O92" s="9" t="n">
-        <v>1.5554</v>
+        <v>1.6905</v>
       </c>
     </row>
     <row r="93">
@@ -4683,34 +4683,34 @@
         </is>
       </c>
       <c r="F93" s="6" t="n">
-        <v>1233298</v>
+        <v>1340440</v>
       </c>
       <c r="G93" s="7" t="n">
         <v>3216.2</v>
       </c>
       <c r="H93" s="8" t="n">
-        <v>396.6533</v>
+        <v>431.1123</v>
       </c>
       <c r="I93" s="7" t="n">
         <v>3216.2</v>
       </c>
       <c r="J93" s="8" t="n">
-        <v>396.6533</v>
+        <v>431.1123</v>
       </c>
       <c r="K93" s="7" t="n">
         <v>3247</v>
       </c>
       <c r="L93" s="8" t="n">
-        <v>400.4519</v>
+        <v>435.2409</v>
       </c>
       <c r="M93" s="9" t="n">
         <v>-0.9486</v>
       </c>
       <c r="N93" s="10" t="n">
-        <v>-0.01453</v>
+        <v>-0.01579</v>
       </c>
       <c r="O93" s="9" t="n">
-        <v>1.5315</v>
+        <v>1.6645</v>
       </c>
     </row>
     <row r="94">
@@ -4738,34 +4738,34 @@
         </is>
       </c>
       <c r="F94" s="6" t="n">
-        <v>14331367</v>
+        <v>15576395</v>
       </c>
       <c r="G94" s="7" t="n">
         <v>255.15</v>
       </c>
       <c r="H94" s="8" t="n">
-        <v>365.6648</v>
+        <v>397.4317</v>
       </c>
       <c r="I94" s="7" t="n">
         <v>255.15</v>
       </c>
       <c r="J94" s="8" t="n">
-        <v>365.6648</v>
+        <v>397.4317</v>
       </c>
       <c r="K94" s="7" t="n">
         <v>256.35</v>
       </c>
       <c r="L94" s="8" t="n">
-        <v>367.3846</v>
+        <v>399.3009</v>
       </c>
       <c r="M94" s="9" t="n">
         <v>-0.4681</v>
       </c>
       <c r="N94" s="10" t="n">
-        <v>-0.00661</v>
+        <v>-0.00718</v>
       </c>
       <c r="O94" s="9" t="n">
-        <v>1.4118</v>
+        <v>1.5345</v>
       </c>
     </row>
     <row r="95">
@@ -4793,34 +4793,34 @@
         </is>
       </c>
       <c r="F95" s="6" t="n">
-        <v>17285110</v>
+        <v>18786742</v>
       </c>
       <c r="G95" s="7" t="n">
         <v>186.45</v>
       </c>
       <c r="H95" s="8" t="n">
-        <v>322.2809</v>
+        <v>350.2788</v>
       </c>
       <c r="I95" s="7" t="n">
         <v>186.45</v>
       </c>
       <c r="J95" s="8" t="n">
-        <v>322.2809</v>
+        <v>350.2788</v>
       </c>
       <c r="K95" s="7" t="n">
         <v>188.37</v>
       </c>
       <c r="L95" s="8" t="n">
-        <v>325.5996</v>
+        <v>353.8859</v>
       </c>
       <c r="M95" s="9" t="n">
         <v>-1.0193</v>
       </c>
       <c r="N95" s="10" t="n">
-        <v>-0.01268</v>
+        <v>-0.01379</v>
       </c>
       <c r="O95" s="9" t="n">
-        <v>1.2443</v>
+        <v>1.3524</v>
       </c>
     </row>
     <row r="96">
@@ -4893,14 +4893,14 @@
       <c r="H97" s="11" t="n"/>
       <c r="I97" s="11" t="n"/>
       <c r="J97" s="13" t="n">
-        <v>2222.663</v>
+        <v>2404.649</v>
       </c>
       <c r="K97" s="11" t="n"/>
       <c r="L97" s="11" t="n"/>
       <c r="M97" s="11" t="n"/>
       <c r="N97" s="11" t="n"/>
       <c r="O97" s="14" t="n">
-        <v>8.58</v>
+        <v>9.279999999999999</v>
       </c>
     </row>
     <row r="98">
@@ -4928,34 +4928,34 @@
         </is>
       </c>
       <c r="F98" s="6" t="n">
-        <v>2009308</v>
+        <v>2183865</v>
       </c>
       <c r="G98" s="7" t="n">
         <v>1850.7</v>
       </c>
       <c r="H98" s="8" t="n">
-        <v>371.8626</v>
+        <v>404.1679</v>
       </c>
       <c r="I98" s="7" t="n">
         <v>1850.7</v>
       </c>
       <c r="J98" s="8" t="n">
-        <v>371.8626</v>
+        <v>404.1679</v>
       </c>
       <c r="K98" s="7" t="n">
         <v>1877.3</v>
       </c>
       <c r="L98" s="8" t="n">
-        <v>377.2074</v>
+        <v>409.977</v>
       </c>
       <c r="M98" s="9" t="n">
         <v>-1.4169</v>
       </c>
       <c r="N98" s="10" t="n">
-        <v>-0.02034</v>
+        <v>-0.02211</v>
       </c>
       <c r="O98" s="9" t="n">
-        <v>1.4358</v>
+        <v>1.5605</v>
       </c>
     </row>
     <row r="99">
@@ -4973,14 +4973,14 @@
       <c r="H99" s="11" t="n"/>
       <c r="I99" s="11" t="n"/>
       <c r="J99" s="13" t="n">
-        <v>371.863</v>
+        <v>404.168</v>
       </c>
       <c r="K99" s="11" t="n"/>
       <c r="L99" s="11" t="n"/>
       <c r="M99" s="11" t="n"/>
       <c r="N99" s="11" t="n"/>
       <c r="O99" s="14" t="n">
-        <v>1.44</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="100">
@@ -5008,34 +5008,34 @@
         </is>
       </c>
       <c r="F100" s="6" t="n">
-        <v>21146739</v>
+        <v>22983847</v>
       </c>
       <c r="G100" s="7" t="n">
         <v>108.44</v>
       </c>
       <c r="H100" s="8" t="n">
-        <v>229.3152</v>
+        <v>249.2368</v>
       </c>
       <c r="I100" s="7" t="n">
         <v>108.44</v>
       </c>
       <c r="J100" s="8" t="n">
-        <v>229.3152</v>
+        <v>249.2368</v>
       </c>
       <c r="K100" s="7" t="n">
         <v>108.07</v>
       </c>
       <c r="L100" s="8" t="n">
-        <v>228.5328</v>
+        <v>248.3864</v>
       </c>
       <c r="M100" s="9" t="n">
         <v>0.3424</v>
       </c>
       <c r="N100" s="10" t="n">
-        <v>0.00303</v>
+        <v>0.00329</v>
       </c>
       <c r="O100" s="9" t="n">
-        <v>0.8854</v>
+        <v>0.9623</v>
       </c>
     </row>
     <row r="101">
@@ -5063,34 +5063,34 @@
         </is>
       </c>
       <c r="F101" s="6" t="n">
-        <v>517626</v>
+        <v>562594</v>
       </c>
       <c r="G101" s="7" t="n">
         <v>1796</v>
       </c>
       <c r="H101" s="8" t="n">
-        <v>92.96559999999999</v>
+        <v>101.0419</v>
       </c>
       <c r="I101" s="7" t="n">
         <v>1796</v>
       </c>
       <c r="J101" s="8" t="n">
-        <v>92.96559999999999</v>
+        <v>101.0419</v>
       </c>
       <c r="K101" s="7" t="n">
         <v>1813.3</v>
       </c>
       <c r="L101" s="8" t="n">
-        <v>93.86109999999999</v>
+        <v>102.0152</v>
       </c>
       <c r="M101" s="9" t="n">
         <v>-0.9540999999999999</v>
       </c>
       <c r="N101" s="10" t="n">
-        <v>-0.00342</v>
+        <v>-0.00372</v>
       </c>
       <c r="O101" s="9" t="n">
-        <v>0.3589</v>
+        <v>0.3901</v>
       </c>
     </row>
     <row r="102">
@@ -5108,14 +5108,14 @@
       <c r="H102" s="11" t="n"/>
       <c r="I102" s="11" t="n"/>
       <c r="J102" s="13" t="n">
-        <v>322.281</v>
+        <v>350.279</v>
       </c>
       <c r="K102" s="11" t="n"/>
       <c r="L102" s="11" t="n"/>
       <c r="M102" s="11" t="n"/>
       <c r="N102" s="11" t="n"/>
       <c r="O102" s="14" t="n">
-        <v>1.24</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="104">
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="C104" s="15" t="n">
-        <v>22824.834</v>
+        <v>24604.905</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -5140,11 +5140,11 @@
         </is>
       </c>
       <c r="C105" s="15" t="n">
-        <v>3075.066</v>
+        <v>1294.995</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>₹cr (11.87%)</t>
+          <t>₹cr (5.0%)</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C108" s="15" t="n">
-        <v>-0.1378</v>
+        <v>-0.1433</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>

</xml_diff>